<commit_message>
Update Goal 1 indicators for 2025-2026
</commit_message>
<xml_diff>
--- a/data/2025_RW-SDG_Data.xlsx
+++ b/data/2025_RW-SDG_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GGessienne\Documents\sdg-data-rwanda\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C798CD4E-6556-4972-832D-C886FC700565}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A5296F9-933B-4D55-B38C-8B6BF9E53BCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14925" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -13912,7 +13912,7 @@
       <c r="AG45" s="9">
         <v>0.24</v>
       </c>
-      <c r="AH45" s="10">
+      <c r="AH45" s="9">
         <v>0.16700000000000001</v>
       </c>
       <c r="AJ45" s="9">
@@ -13921,7 +13921,7 @@
       <c r="AM45" s="9">
         <v>0.15</v>
       </c>
-      <c r="AR45" s="10">
+      <c r="AR45" s="9">
         <v>0.129</v>
       </c>
       <c r="AT45" s="10">
@@ -13974,7 +13974,7 @@
       <c r="AG46" s="9">
         <v>0.09</v>
       </c>
-      <c r="AH46" s="10">
+      <c r="AH46" s="9">
         <v>6.5000000000000002E-2</v>
       </c>
       <c r="AJ46" s="9">
@@ -13983,7 +13983,7 @@
       <c r="AM46" s="9">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="AR46" s="10">
+      <c r="AR46" s="9">
         <v>5.6000000000000001E-2</v>
       </c>
       <c r="AT46" s="10">
@@ -14036,7 +14036,7 @@
       <c r="AG47" s="9">
         <v>0.27</v>
       </c>
-      <c r="AH47" s="10">
+      <c r="AH47" s="9">
         <v>0.187</v>
       </c>
       <c r="AJ47" s="9">
@@ -14045,7 +14045,7 @@
       <c r="AM47" s="9">
         <v>0.17</v>
       </c>
-      <c r="AR47" s="10">
+      <c r="AR47" s="9">
         <v>0.159</v>
       </c>
       <c r="AT47" s="10">
@@ -14098,7 +14098,7 @@
       <c r="AG48" s="9">
         <v>0.12</v>
       </c>
-      <c r="AH48" s="10">
+      <c r="AH48" s="9">
         <v>6.4000000000000001E-2</v>
       </c>
       <c r="AJ48" s="9">
@@ -14107,7 +14107,7 @@
       <c r="AM48" s="9">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="AR48" s="10">
+      <c r="AR48" s="9">
         <v>0.04</v>
       </c>
       <c r="AT48" s="10">
@@ -14160,7 +14160,7 @@
       <c r="AG49" s="9">
         <v>0.28999999999999998</v>
       </c>
-      <c r="AH49" s="10">
+      <c r="AH49" s="9">
         <v>0.17100000000000001</v>
       </c>
       <c r="AJ49" s="9">
@@ -14169,7 +14169,7 @@
       <c r="AM49" s="9">
         <v>0.19</v>
       </c>
-      <c r="AR49" s="10">
+      <c r="AR49" s="9">
         <v>0.14899999999999999</v>
       </c>
       <c r="AT49" s="10">
@@ -14222,7 +14222,7 @@
       <c r="AG50" s="9">
         <v>0.25</v>
       </c>
-      <c r="AH50" s="10">
+      <c r="AH50" s="9">
         <v>0.189</v>
       </c>
       <c r="AJ50" s="9">
@@ -14231,7 +14231,7 @@
       <c r="AM50" s="9">
         <v>0.16</v>
       </c>
-      <c r="AR50" s="10">
+      <c r="AR50" s="9">
         <v>0.15</v>
       </c>
       <c r="AT50" s="10">
@@ -14284,7 +14284,7 @@
       <c r="AG51" s="9">
         <v>0.18</v>
       </c>
-      <c r="AH51" s="10">
+      <c r="AH51" s="9">
         <v>0.161</v>
       </c>
       <c r="AJ51" s="9">
@@ -14293,7 +14293,7 @@
       <c r="AM51" s="9">
         <v>0.11</v>
       </c>
-      <c r="AR51" s="10">
+      <c r="AR51" s="9">
         <v>0.122</v>
       </c>
       <c r="AT51" s="10">
@@ -14346,7 +14346,7 @@
       <c r="AG52" s="9">
         <v>0.26</v>
       </c>
-      <c r="AH52" s="10">
+      <c r="AH52" s="9">
         <v>0.192</v>
       </c>
       <c r="AJ52" s="9">
@@ -14355,7 +14355,7 @@
       <c r="AM52" s="9">
         <v>0.17</v>
       </c>
-      <c r="AR52" s="10">
+      <c r="AR52" s="9">
         <v>0.15</v>
       </c>
       <c r="AT52" s="10">
@@ -15057,7 +15057,7 @@
         <v>53.7</v>
       </c>
     </row>
-    <row r="65" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="65" spans="1:47" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A65" t="s">
         <v>51</v>
       </c>
@@ -15116,7 +15116,7 @@
         <v>75.8</v>
       </c>
     </row>
-    <row r="66" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="66" spans="1:47" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A66" t="s">
         <v>51</v>
       </c>
@@ -15169,7 +15169,7 @@
         <v>77.599999999999994</v>
       </c>
     </row>
-    <row r="67" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="67" spans="1:47" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A67" t="s">
         <v>51</v>
       </c>
@@ -15243,7 +15243,7 @@
         <v>99.07</v>
       </c>
     </row>
-    <row r="68" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="68" spans="1:47" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A68" t="s">
         <v>129</v>
       </c>
@@ -15302,7 +15302,7 @@
         <v>81.2</v>
       </c>
     </row>
-    <row r="69" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="69" spans="1:47" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A69" t="s">
         <v>129</v>
       </c>
@@ -15361,7 +15361,7 @@
         <v>79.2</v>
       </c>
     </row>
-    <row r="70" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="70" spans="1:47" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A70" t="s">
         <v>129</v>
       </c>
@@ -15420,7 +15420,7 @@
         <v>82.7</v>
       </c>
     </row>
-    <row r="71" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="71" spans="1:47" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A71" t="s">
         <v>131</v>
       </c>
@@ -15466,7 +15466,7 @@
       <c r="AM71">
         <v>0.69</v>
       </c>
-      <c r="AN71">
+      <c r="AN71" s="9">
         <v>2.1</v>
       </c>
       <c r="AO71">
@@ -15475,20 +15475,23 @@
       <c r="AP71">
         <v>2.35</v>
       </c>
-      <c r="AQ71">
+      <c r="AQ71" s="9">
         <v>0.9</v>
       </c>
       <c r="AR71">
         <v>1.55</v>
       </c>
-      <c r="AS71">
+      <c r="AS71" s="9">
         <v>1.8</v>
       </c>
       <c r="AT71">
         <v>1.38</v>
       </c>
-    </row>
-    <row r="72" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="AU71">
+        <v>1.03</v>
+      </c>
+    </row>
+    <row r="72" spans="1:47" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A72" t="s">
         <v>131</v>
       </c>
@@ -15555,8 +15558,11 @@
       <c r="AT72">
         <v>3.25</v>
       </c>
-    </row>
-    <row r="73" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="AU72">
+        <v>2.0299999999999998</v>
+      </c>
+    </row>
+    <row r="73" spans="1:47" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A73" t="s">
         <v>849</v>
       </c>
@@ -15617,8 +15623,11 @@
       <c r="AT73">
         <v>2005</v>
       </c>
-    </row>
-    <row r="74" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="AU73">
+        <v>1841</v>
+      </c>
+    </row>
+    <row r="74" spans="1:47" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A74" t="s">
         <v>849</v>
       </c>
@@ -15679,8 +15688,11 @@
       <c r="AT74">
         <v>1355.3</v>
       </c>
-    </row>
-    <row r="75" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="AU74">
+        <v>1155</v>
+      </c>
+    </row>
+    <row r="75" spans="1:47" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A75" t="s">
         <v>849</v>
       </c>
@@ -15741,8 +15753,11 @@
       <c r="AT75">
         <v>81</v>
       </c>
-    </row>
-    <row r="76" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="AU75">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="76" spans="1:47" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A76" t="s">
         <v>849</v>
       </c>
@@ -15803,8 +15818,11 @@
       <c r="AT76">
         <v>2</v>
       </c>
-    </row>
-    <row r="77" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="AU76">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="77" spans="1:47" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A77" t="s">
         <v>849</v>
       </c>
@@ -15865,8 +15883,11 @@
       <c r="AT77">
         <v>42</v>
       </c>
-    </row>
-    <row r="78" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="AU77">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="78" spans="1:47" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A78" t="s">
         <v>849</v>
       </c>
@@ -15927,8 +15948,11 @@
       <c r="AT78">
         <v>11</v>
       </c>
-    </row>
-    <row r="79" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="AU78">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="79" spans="1:47" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A79" t="s">
         <v>849</v>
       </c>
@@ -15989,8 +16013,11 @@
       <c r="AT79">
         <v>34</v>
       </c>
-    </row>
-    <row r="80" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="AU79">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="80" spans="1:47" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A80" t="s">
         <v>849</v>
       </c>
@@ -16225,6 +16252,9 @@
       <c r="AT83">
         <v>306</v>
       </c>
+      <c r="AU83">
+        <v>58</v>
+      </c>
     </row>
     <row r="84" spans="1:48" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A84" t="s">
@@ -16284,6 +16314,9 @@
       <c r="AT84">
         <v>12</v>
       </c>
+      <c r="AU84">
+        <v>9</v>
+      </c>
     </row>
     <row r="85" spans="1:48" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A85" t="s">
@@ -16343,6 +16376,9 @@
       <c r="AT85">
         <v>69</v>
       </c>
+      <c r="AU85">
+        <v>25</v>
+      </c>
     </row>
     <row r="86" spans="1:48" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A86" t="s">
@@ -16402,6 +16438,9 @@
       <c r="AT86">
         <v>3146</v>
       </c>
+      <c r="AU86">
+        <v>104</v>
+      </c>
     </row>
     <row r="87" spans="1:48" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A87" t="s">
@@ -16465,6 +16504,12 @@
         <v>100</v>
       </c>
       <c r="AT87">
+        <v>100</v>
+      </c>
+      <c r="AU87">
+        <v>100</v>
+      </c>
+      <c r="AV87">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update indicators 2.1.1, 2.1.2
</commit_message>
<xml_diff>
--- a/data/2025_RW-SDG_Data.xlsx
+++ b/data/2025_RW-SDG_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GGessienne\Documents\sdg-data-rwanda\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A5296F9-933B-4D55-B38C-8B6BF9E53BCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54C536CD-E7E8-4676-8A1D-2FFB3A20C98E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14925" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -17212,22 +17212,31 @@
         <v>89</v>
       </c>
       <c r="AM96">
-        <v>33</v>
+        <v>38.299999999999997</v>
       </c>
       <c r="AN96">
-        <v>32</v>
+        <v>37.6</v>
       </c>
       <c r="AO96">
-        <v>34</v>
+        <v>40.200000000000003</v>
       </c>
       <c r="AP96">
-        <v>32</v>
+        <v>38.799999999999997</v>
       </c>
       <c r="AQ96">
-        <v>32</v>
+        <v>38.5</v>
       </c>
       <c r="AR96">
-        <v>29</v>
+        <v>35.299999999999997</v>
+      </c>
+      <c r="AS96">
+        <v>32.700000000000003</v>
+      </c>
+      <c r="AT96">
+        <v>31.3</v>
+      </c>
+      <c r="AU96">
+        <v>29.9</v>
       </c>
     </row>
     <row r="97" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">

</xml_diff>

<commit_message>
Update DSD for new indicators
</commit_message>
<xml_diff>
--- a/data/2025_RW-SDG_Data.xlsx
+++ b/data/2025_RW-SDG_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GGessienne\Documents\sdg-data-rwanda\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59895DAC-7F3D-4598-8F28-FC3AD4712547}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57CA1C6A-EEA5-46F6-BEF9-6BDA11FD5401}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3503,9 +3503,6 @@
     <t>SH_MDD_CHLD</t>
   </si>
   <si>
-    <t>SH_MDD_WMN_NPRG</t>
-  </si>
-  <si>
     <t>Prevalence of minimum dietary diversity among children aged 6-23 months</t>
   </si>
   <si>
@@ -3515,7 +3512,10 @@
     <t>&lt;2</t>
   </si>
   <si>
-    <t xml:space="preserve">Prevalence of minimum dietary diversity among women aged 15-49 years </t>
+    <t>SH_MDD_WMN</t>
+  </si>
+  <si>
+    <t>Prevalence of minimum dietary diversity among women aged 15-49 years</t>
   </si>
 </sst>
 </file>
@@ -17982,76 +17982,76 @@
       <c r="U108" t="s">
         <v>14</v>
       </c>
-      <c r="V108">
+      <c r="V108" s="7">
         <v>21.1</v>
       </c>
-      <c r="W108">
+      <c r="W108" s="7">
         <v>20.2</v>
       </c>
-      <c r="X108">
+      <c r="X108" s="7">
         <v>19.399999999999999</v>
       </c>
-      <c r="Y108">
+      <c r="Y108" s="7">
         <v>18.600000000000001</v>
       </c>
-      <c r="Z108">
+      <c r="Z108" s="7">
         <v>17.899999999999999</v>
       </c>
-      <c r="AA108">
+      <c r="AA108" s="7">
         <v>17.2</v>
       </c>
-      <c r="AB108">
+      <c r="AB108" s="7">
         <v>16.5</v>
       </c>
-      <c r="AC108">
+      <c r="AC108" s="7">
         <v>15.9</v>
       </c>
-      <c r="AD108">
+      <c r="AD108" s="7">
         <v>15.3</v>
       </c>
-      <c r="AE108">
+      <c r="AE108" s="7">
         <v>14.8</v>
       </c>
-      <c r="AF108">
+      <c r="AF108" s="7">
         <v>14.4</v>
       </c>
-      <c r="AG108">
+      <c r="AG108" s="7">
         <v>14.2</v>
       </c>
-      <c r="AH108">
+      <c r="AH108" s="7">
         <v>14.1</v>
       </c>
-      <c r="AI108">
+      <c r="AI108" s="7">
         <v>14.1</v>
       </c>
-      <c r="AJ108">
+      <c r="AJ108" s="7">
         <v>14.2</v>
       </c>
-      <c r="AK108">
+      <c r="AK108" s="7">
         <v>14.3</v>
       </c>
-      <c r="AL108">
+      <c r="AL108" s="7">
         <v>14.4</v>
       </c>
-      <c r="AM108">
+      <c r="AM108" s="7">
         <v>14.4</v>
       </c>
-      <c r="AN108">
+      <c r="AN108" s="7">
         <v>14.5</v>
       </c>
-      <c r="AO108">
+      <c r="AO108" s="7">
         <v>14.6</v>
       </c>
-      <c r="AP108">
+      <c r="AP108" s="7">
         <v>14.7</v>
       </c>
-      <c r="AQ108">
+      <c r="AQ108" s="7">
         <v>15</v>
       </c>
-      <c r="AR108">
+      <c r="AR108" s="7">
         <v>15.4</v>
       </c>
-      <c r="AS108">
+      <c r="AS108" s="7">
         <v>16.100000000000001</v>
       </c>
       <c r="AU108" s="7"/>
@@ -18102,76 +18102,76 @@
       <c r="U109" t="s">
         <v>14</v>
       </c>
-      <c r="V109">
+      <c r="V109" s="7">
         <v>20.100000000000001</v>
       </c>
-      <c r="W109">
+      <c r="W109" s="7">
         <v>19.2</v>
       </c>
-      <c r="X109">
+      <c r="X109" s="7">
         <v>18.399999999999999</v>
       </c>
-      <c r="Y109">
+      <c r="Y109" s="7">
         <v>17.7</v>
       </c>
-      <c r="Z109">
+      <c r="Z109" s="7">
         <v>17</v>
       </c>
-      <c r="AA109">
+      <c r="AA109" s="7">
         <v>16.3</v>
       </c>
-      <c r="AB109">
+      <c r="AB109" s="7">
         <v>15.6</v>
       </c>
-      <c r="AC109">
+      <c r="AC109" s="7">
         <v>15</v>
       </c>
-      <c r="AD109">
+      <c r="AD109" s="7">
         <v>14.5</v>
       </c>
-      <c r="AE109">
+      <c r="AE109" s="7">
         <v>14</v>
       </c>
-      <c r="AF109">
+      <c r="AF109" s="7">
         <v>13.6</v>
       </c>
-      <c r="AG109">
+      <c r="AG109" s="7">
         <v>13.4</v>
       </c>
-      <c r="AH109">
+      <c r="AH109" s="7">
         <v>13.3</v>
       </c>
-      <c r="AI109">
+      <c r="AI109" s="7">
         <v>13.3</v>
       </c>
-      <c r="AJ109">
+      <c r="AJ109" s="7">
         <v>13.4</v>
       </c>
-      <c r="AK109">
+      <c r="AK109" s="7">
         <v>13.5</v>
       </c>
-      <c r="AL109">
+      <c r="AL109" s="7">
         <v>13.6</v>
       </c>
-      <c r="AM109">
+      <c r="AM109" s="7">
         <v>13.7</v>
       </c>
-      <c r="AN109">
+      <c r="AN109" s="7">
         <v>13.8</v>
       </c>
-      <c r="AO109">
+      <c r="AO109" s="7">
         <v>13.9</v>
       </c>
-      <c r="AP109">
+      <c r="AP109" s="7">
         <v>14.1</v>
       </c>
-      <c r="AQ109">
+      <c r="AQ109" s="7">
         <v>14.4</v>
       </c>
-      <c r="AR109">
+      <c r="AR109" s="7">
         <v>14.8</v>
       </c>
-      <c r="AS109">
+      <c r="AS109" s="7">
         <v>15.5</v>
       </c>
       <c r="AU109" s="7"/>
@@ -18222,76 +18222,76 @@
       <c r="U110" t="s">
         <v>14</v>
       </c>
-      <c r="V110">
+      <c r="V110" s="7">
         <v>29.8</v>
       </c>
-      <c r="W110">
+      <c r="W110" s="7">
         <v>28.9</v>
       </c>
-      <c r="X110">
+      <c r="X110" s="7">
         <v>28</v>
       </c>
-      <c r="Y110">
+      <c r="Y110" s="7">
         <v>27.2</v>
       </c>
-      <c r="Z110">
+      <c r="Z110" s="7">
         <v>26.4</v>
       </c>
-      <c r="AA110">
+      <c r="AA110" s="7">
         <v>25.5</v>
       </c>
-      <c r="AB110">
+      <c r="AB110" s="7">
         <v>24.8</v>
       </c>
-      <c r="AC110">
+      <c r="AC110" s="7">
         <v>24</v>
       </c>
-      <c r="AD110">
+      <c r="AD110" s="7">
         <v>23.4</v>
       </c>
-      <c r="AE110">
+      <c r="AE110" s="7">
         <v>22.9</v>
       </c>
-      <c r="AF110">
+      <c r="AF110" s="7">
         <v>22.5</v>
       </c>
-      <c r="AG110">
+      <c r="AG110" s="7">
         <v>22.3</v>
       </c>
-      <c r="AH110">
+      <c r="AH110" s="7">
         <v>22.3</v>
       </c>
-      <c r="AI110">
+      <c r="AI110" s="7">
         <v>22.4</v>
       </c>
-      <c r="AJ110">
+      <c r="AJ110" s="7">
         <v>22.5</v>
       </c>
-      <c r="AK110">
+      <c r="AK110" s="7">
         <v>22.6</v>
       </c>
-      <c r="AL110">
+      <c r="AL110" s="7">
         <v>22.7</v>
       </c>
-      <c r="AM110">
+      <c r="AM110" s="7">
         <v>22.8</v>
       </c>
-      <c r="AN110">
+      <c r="AN110" s="7">
         <v>22.8</v>
       </c>
-      <c r="AO110">
+      <c r="AO110" s="7">
         <v>22.9</v>
       </c>
-      <c r="AP110">
+      <c r="AP110" s="7">
         <v>23</v>
       </c>
-      <c r="AQ110">
+      <c r="AQ110" s="7">
         <v>23.2</v>
       </c>
-      <c r="AR110">
+      <c r="AR110" s="7">
         <v>23.5</v>
       </c>
-      <c r="AS110">
+      <c r="AS110" s="7">
         <v>23.9</v>
       </c>
       <c r="AU110" s="7"/>
@@ -18328,13 +18328,13 @@
         <v>1106</v>
       </c>
       <c r="P111" t="s">
+        <v>1125</v>
+      </c>
+      <c r="R111" t="s">
         <v>1126</v>
       </c>
-      <c r="R111" t="s">
+      <c r="S111" t="s">
         <v>1127</v>
-      </c>
-      <c r="S111" t="s">
-        <v>1128</v>
       </c>
       <c r="T111" t="s">
         <v>89</v>
@@ -18361,7 +18361,7 @@
         <v>1123</v>
       </c>
       <c r="C112" t="s">
-        <v>1125</v>
+        <v>1128</v>
       </c>
       <c r="D112" t="s">
         <v>89</v>

</xml_diff>